<commit_message>
licence and variable name update
</commit_message>
<xml_diff>
--- a/projeto_maturacao/data/raw/dados_maturidade.xlsx
+++ b/projeto_maturacao/data/raw/dados_maturidade.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="23801"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diogo Silva\Documents\GitHub\tese_cap3\projeto_maturacao\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\nuptial_manuscript\projeto_maturacao\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116BF1FF-3EB1-41B6-9E56-1B614815F860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F073465-ADC6-4956-A9A8-0C7DED30A755}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="362">
   <si>
     <t>ID</t>
   </si>
@@ -911,9 +909,6 @@
     <t>Female</t>
   </si>
   <si>
-    <t>Residencia</t>
-  </si>
-  <si>
     <t>F97</t>
   </si>
   <si>
@@ -939,12 +934,6 @@
   </si>
   <si>
     <t>F105</t>
-  </si>
-  <si>
-    <t>Wandering</t>
-  </si>
-  <si>
-    <t>Resident</t>
   </si>
   <si>
     <t>F106</t>
@@ -1198,7 +1187,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1494,16 +1483,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J168"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I168"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="8" width="12.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="7" width="8.90625" style="1"/>
+    <col min="8" max="8" width="12.90625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="11.453125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,13 +1517,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1560,11 +1545,11 @@
       <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="2">
+      <c r="I2" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1583,11 +1568,11 @@
       <c r="H3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="2">
+      <c r="I3" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -1612,11 +1597,11 @@
       <c r="H4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="2">
+      <c r="I4" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1641,11 +1626,11 @@
       <c r="H5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="2">
+      <c r="I5" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
@@ -1670,11 +1655,11 @@
       <c r="H6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="2">
+      <c r="I6" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>33</v>
       </c>
@@ -1699,11 +1684,11 @@
       <c r="H7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="2">
+      <c r="I7" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
@@ -1728,11 +1713,11 @@
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="2">
+      <c r="I8" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -1757,11 +1742,11 @@
       <c r="H9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="2">
+      <c r="I9" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -1786,11 +1771,11 @@
       <c r="H10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="2">
+      <c r="I10" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>52</v>
       </c>
@@ -1815,11 +1800,11 @@
       <c r="H11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="2">
+      <c r="I11" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>57</v>
       </c>
@@ -1844,11 +1829,11 @@
       <c r="H12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="2">
+      <c r="I12" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>60</v>
       </c>
@@ -1873,11 +1858,11 @@
       <c r="H13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="2">
+      <c r="I13" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>62</v>
       </c>
@@ -1902,11 +1887,11 @@
       <c r="H14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="2">
+      <c r="I14" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>67</v>
       </c>
@@ -1931,11 +1916,11 @@
       <c r="H15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="2">
+      <c r="I15" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>71</v>
       </c>
@@ -1960,11 +1945,11 @@
       <c r="H16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="2">
+      <c r="I16" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>73</v>
       </c>
@@ -1989,11 +1974,11 @@
       <c r="H17" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="2">
+      <c r="I17" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>78</v>
       </c>
@@ -2018,11 +2003,11 @@
       <c r="H18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="2">
+      <c r="I18" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>80</v>
       </c>
@@ -2047,11 +2032,11 @@
       <c r="H19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J19" s="2">
+      <c r="I19" s="2">
         <v>45066</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>83</v>
       </c>
@@ -2076,11 +2061,11 @@
       <c r="H20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J20" s="2">
+      <c r="I20" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>85</v>
       </c>
@@ -2105,11 +2090,11 @@
       <c r="H21" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J21" s="2">
+      <c r="I21" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>88</v>
       </c>
@@ -2134,11 +2119,11 @@
       <c r="H22" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J22" s="2">
+      <c r="I22" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>91</v>
       </c>
@@ -2163,11 +2148,11 @@
       <c r="H23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J23" s="2">
+      <c r="I23" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>93</v>
       </c>
@@ -2192,11 +2177,11 @@
       <c r="H24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J24" s="2">
+      <c r="I24" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>96</v>
       </c>
@@ -2221,11 +2206,11 @@
       <c r="H25" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J25" s="2">
+      <c r="I25" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>99</v>
       </c>
@@ -2250,11 +2235,11 @@
       <c r="H26" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J26" s="2">
+      <c r="I26" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>101</v>
       </c>
@@ -2279,11 +2264,11 @@
       <c r="H27" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J27" s="2">
+      <c r="I27" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>103</v>
       </c>
@@ -2308,11 +2293,11 @@
       <c r="H28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J28" s="2">
+      <c r="I28" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>105</v>
       </c>
@@ -2337,11 +2322,11 @@
       <c r="H29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J29" s="2">
+      <c r="I29" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>107</v>
       </c>
@@ -2366,11 +2351,11 @@
       <c r="H30" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J30" s="2">
+      <c r="I30" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>108</v>
       </c>
@@ -2395,11 +2380,11 @@
       <c r="H31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J31" s="2">
+      <c r="I31" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>110</v>
       </c>
@@ -2424,11 +2409,11 @@
       <c r="H32" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J32" s="2">
+      <c r="I32" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>111</v>
       </c>
@@ -2453,11 +2438,11 @@
       <c r="H33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J33" s="2">
+      <c r="I33" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>115</v>
       </c>
@@ -2482,11 +2467,11 @@
       <c r="H34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="2">
+      <c r="I34" s="2">
         <v>45067</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>117</v>
       </c>
@@ -2511,11 +2496,11 @@
       <c r="H35" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J35" s="2">
+      <c r="I35" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>122</v>
       </c>
@@ -2540,11 +2525,11 @@
       <c r="H36" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J36" s="2">
+      <c r="I36" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>125</v>
       </c>
@@ -2569,11 +2554,11 @@
       <c r="H37" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J37" s="2">
+      <c r="I37" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>130</v>
       </c>
@@ -2598,11 +2583,11 @@
       <c r="H38" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J38" s="2">
+      <c r="I38" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>135</v>
       </c>
@@ -2627,11 +2612,11 @@
       <c r="H39" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J39" s="2">
+      <c r="I39" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>140</v>
       </c>
@@ -2656,11 +2641,11 @@
       <c r="H40" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J40" s="2">
+      <c r="I40" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>145</v>
       </c>
@@ -2685,11 +2670,11 @@
       <c r="H41" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J41" s="2">
+      <c r="I41" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>150</v>
       </c>
@@ -2714,11 +2699,11 @@
       <c r="H42" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J42" s="2">
+      <c r="I42" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>155</v>
       </c>
@@ -2743,11 +2728,11 @@
       <c r="H43" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J43" s="2">
+      <c r="I43" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>158</v>
       </c>
@@ -2772,11 +2757,11 @@
       <c r="H44" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J44" s="2">
+      <c r="I44" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>163</v>
       </c>
@@ -2801,11 +2786,11 @@
       <c r="H45" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J45" s="2">
+      <c r="I45" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>168</v>
       </c>
@@ -2830,11 +2815,11 @@
       <c r="H46" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J46" s="2">
+      <c r="I46" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>173</v>
       </c>
@@ -2859,11 +2844,11 @@
       <c r="H47" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J47" s="2">
+      <c r="I47" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>177</v>
       </c>
@@ -2888,11 +2873,11 @@
       <c r="H48" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J48" s="2">
+      <c r="I48" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>182</v>
       </c>
@@ -2917,11 +2902,11 @@
       <c r="H49" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J49" s="2">
+      <c r="I49" s="2">
         <v>45082</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>187</v>
       </c>
@@ -2946,11 +2931,11 @@
       <c r="H50" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J50" s="2">
+      <c r="I50" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>191</v>
       </c>
@@ -2975,11 +2960,11 @@
       <c r="H51" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J51" s="2">
+      <c r="I51" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>195</v>
       </c>
@@ -3004,11 +2989,11 @@
       <c r="H52" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J52" s="2">
+      <c r="I52" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>199</v>
       </c>
@@ -3033,11 +3018,11 @@
       <c r="H53" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J53" s="2">
+      <c r="I53" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>204</v>
       </c>
@@ -3062,11 +3047,11 @@
       <c r="H54" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J54" s="2">
+      <c r="I54" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>209</v>
       </c>
@@ -3091,11 +3076,11 @@
       <c r="H55" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J55" s="2">
+      <c r="I55" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>214</v>
       </c>
@@ -3120,11 +3105,11 @@
       <c r="H56" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J56" s="2">
+      <c r="I56" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>219</v>
       </c>
@@ -3149,11 +3134,11 @@
       <c r="H57" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J57" s="2">
+      <c r="I57" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>223</v>
       </c>
@@ -3178,11 +3163,11 @@
       <c r="H58" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J58" s="2">
+      <c r="I58" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>227</v>
       </c>
@@ -3207,11 +3192,11 @@
       <c r="H59" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J59" s="2">
+      <c r="I59" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>232</v>
       </c>
@@ -3236,11 +3221,11 @@
       <c r="H60" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J60" s="2">
+      <c r="I60" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>237</v>
       </c>
@@ -3265,11 +3250,11 @@
       <c r="H61" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J61" s="2">
+      <c r="I61" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>242</v>
       </c>
@@ -3294,11 +3279,11 @@
       <c r="H62" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J62" s="2">
+      <c r="I62" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>246</v>
       </c>
@@ -3323,11 +3308,11 @@
       <c r="H63" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J63" s="2">
+      <c r="I63" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>251</v>
       </c>
@@ -3352,11 +3337,11 @@
       <c r="H64" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J64" s="2">
+      <c r="I64" s="2">
         <v>45083</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>255</v>
       </c>
@@ -3381,11 +3366,11 @@
       <c r="H65" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J65" s="2">
+      <c r="I65" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>256</v>
       </c>
@@ -3410,11 +3395,11 @@
       <c r="H66" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J66" s="2">
+      <c r="I66" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>257</v>
       </c>
@@ -3439,11 +3424,11 @@
       <c r="H67" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J67" s="2">
+      <c r="I67" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>258</v>
       </c>
@@ -3468,11 +3453,11 @@
       <c r="H68" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J68" s="2">
+      <c r="I68" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>259</v>
       </c>
@@ -3497,11 +3482,11 @@
       <c r="H69" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J69" s="2">
+      <c r="I69" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>260</v>
       </c>
@@ -3526,11 +3511,11 @@
       <c r="H70" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J70" s="2">
+      <c r="I70" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>261</v>
       </c>
@@ -3555,11 +3540,11 @@
       <c r="H71" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J71" s="2">
+      <c r="I71" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>262</v>
       </c>
@@ -3584,11 +3569,11 @@
       <c r="H72" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J72" s="2">
+      <c r="I72" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>263</v>
       </c>
@@ -3613,11 +3598,11 @@
       <c r="H73" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J73" s="2">
+      <c r="I73" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>264</v>
       </c>
@@ -3642,11 +3627,11 @@
       <c r="H74" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J74" s="2">
+      <c r="I74" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>265</v>
       </c>
@@ -3671,11 +3656,11 @@
       <c r="H75" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J75" s="2">
+      <c r="I75" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>266</v>
       </c>
@@ -3700,11 +3685,11 @@
       <c r="H76" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J76" s="2">
+      <c r="I76" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>267</v>
       </c>
@@ -3729,11 +3714,11 @@
       <c r="H77" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J77" s="2">
+      <c r="I77" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>268</v>
       </c>
@@ -3758,11 +3743,11 @@
       <c r="H78" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J78" s="2">
+      <c r="I78" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>269</v>
       </c>
@@ -3787,11 +3772,11 @@
       <c r="H79" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J79" s="2">
+      <c r="I79" s="2">
         <v>45096</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>270</v>
       </c>
@@ -3816,11 +3801,11 @@
       <c r="H80" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J80" s="2">
+      <c r="I80" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>271</v>
       </c>
@@ -3845,11 +3830,11 @@
       <c r="H81" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J81" s="2">
+      <c r="I81" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>272</v>
       </c>
@@ -3874,11 +3859,11 @@
       <c r="H82" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J82" s="2">
+      <c r="I82" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>273</v>
       </c>
@@ -3903,11 +3888,11 @@
       <c r="H83" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J83" s="2">
+      <c r="I83" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>274</v>
       </c>
@@ -3932,11 +3917,11 @@
       <c r="H84" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J84" s="2">
+      <c r="I84" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>275</v>
       </c>
@@ -3961,11 +3946,11 @@
       <c r="H85" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J85" s="2">
+      <c r="I85" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>276</v>
       </c>
@@ -3990,11 +3975,11 @@
       <c r="H86" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J86" s="2">
+      <c r="I86" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>277</v>
       </c>
@@ -4019,11 +4004,11 @@
       <c r="H87" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J87" s="2">
+      <c r="I87" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>278</v>
       </c>
@@ -4048,11 +4033,11 @@
       <c r="H88" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J88" s="2">
+      <c r="I88" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>279</v>
       </c>
@@ -4077,11 +4062,11 @@
       <c r="H89" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J89" s="2">
+      <c r="I89" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>280</v>
       </c>
@@ -4106,11 +4091,11 @@
       <c r="H90" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J90" s="2">
+      <c r="I90" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>281</v>
       </c>
@@ -4135,11 +4120,11 @@
       <c r="H91" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J91" s="2">
+      <c r="I91" s="2">
         <v>45097</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>282</v>
       </c>
@@ -4158,14 +4143,11 @@
       <c r="H92" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I92" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J92" s="2">
+      <c r="I92" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>283</v>
       </c>
@@ -4184,14 +4166,11 @@
       <c r="H93" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I93" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J93" s="2">
+      <c r="I93" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>284</v>
       </c>
@@ -4210,14 +4189,11 @@
       <c r="H94" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I94" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J94" s="2">
+      <c r="I94" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>285</v>
       </c>
@@ -4236,14 +4212,11 @@
       <c r="H95" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I95" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J95" s="2">
+      <c r="I95" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>286</v>
       </c>
@@ -4262,14 +4235,11 @@
       <c r="H96" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I96" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J96" s="2">
+      <c r="I96" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>287</v>
       </c>
@@ -4288,16 +4258,13 @@
       <c r="H97" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I97" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J97" s="2">
+      <c r="I97" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>290</v>
@@ -4314,16 +4281,13 @@
       <c r="H98" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I98" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J98" s="2">
+      <c r="I98" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>290</v>
@@ -4340,16 +4304,13 @@
       <c r="H99" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I99" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J99" s="2">
+      <c r="I99" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>290</v>
@@ -4366,16 +4327,13 @@
       <c r="H100" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I100" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J100" s="2">
+      <c r="I100" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>290</v>
@@ -4392,16 +4350,13 @@
       <c r="H101" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I101" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J101" s="2">
+      <c r="I101" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>290</v>
@@ -4418,16 +4373,13 @@
       <c r="H102" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I102" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J102" s="2">
+      <c r="I102" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>290</v>
@@ -4444,16 +4396,13 @@
       <c r="H103" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I103" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J103" s="2">
+      <c r="I103" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>290</v>
@@ -4470,16 +4419,13 @@
       <c r="H104" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I104" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J104" s="2">
+      <c r="I104" s="2">
         <v>45098</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>290</v>
@@ -4496,16 +4442,13 @@
       <c r="H105" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I105" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J105" s="2">
+      <c r="I105" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>290</v>
@@ -4522,16 +4465,13 @@
       <c r="H106" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I106" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J106" s="2">
+      <c r="I106" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>290</v>
@@ -4548,16 +4488,13 @@
       <c r="H107" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I107" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J107" s="2">
+      <c r="I107" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>290</v>
@@ -4574,16 +4511,13 @@
       <c r="H108" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I108" s="1" t="s">
+      <c r="I108" s="2">
+        <v>45108</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A109" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="J108" s="2">
-        <v>45108</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A109" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>290</v>
@@ -4600,16 +4534,13 @@
       <c r="H109" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I109" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J109" s="2">
+      <c r="I109" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>290</v>
@@ -4626,16 +4557,13 @@
       <c r="H110" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I110" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J110" s="2">
+      <c r="I110" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B111" s="1" t="s">
         <v>290</v>
@@ -4652,16 +4580,13 @@
       <c r="H111" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I111" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J111" s="2">
+      <c r="I111" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>290</v>
@@ -4678,16 +4603,13 @@
       <c r="H112" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I112" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J112" s="2">
+      <c r="I112" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>290</v>
@@ -4704,16 +4626,13 @@
       <c r="H113" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I113" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J113" s="2">
+      <c r="I113" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>290</v>
@@ -4730,16 +4649,13 @@
       <c r="H114" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I114" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J114" s="2">
+      <c r="I114" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>290</v>
@@ -4756,16 +4672,13 @@
       <c r="H115" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I115" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J115" s="2">
+      <c r="I115" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>290</v>
@@ -4782,16 +4695,13 @@
       <c r="H116" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I116" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J116" s="2">
+      <c r="I116" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>290</v>
@@ -4808,16 +4718,13 @@
       <c r="H117" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I117" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J117" s="2">
+      <c r="I117" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>290</v>
@@ -4834,16 +4741,13 @@
       <c r="H118" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I118" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J118" s="2">
+      <c r="I118" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>290</v>
@@ -4860,16 +4764,13 @@
       <c r="H119" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I119" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J119" s="2">
+      <c r="I119" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>290</v>
@@ -4886,16 +4787,13 @@
       <c r="H120" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I120" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J120" s="2">
+      <c r="I120" s="2">
         <v>45108</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>290</v>
@@ -4912,16 +4810,13 @@
       <c r="H121" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I121" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J121" s="2">
+      <c r="I121" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B122" s="1" t="s">
         <v>290</v>
@@ -4938,16 +4833,13 @@
       <c r="H122" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I122" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J122" s="2">
+      <c r="I122" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>290</v>
@@ -4964,16 +4856,13 @@
       <c r="H123" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I123" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J123" s="2">
+      <c r="I123" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B124" s="1" t="s">
         <v>290</v>
@@ -4990,16 +4879,13 @@
       <c r="H124" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I124" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J124" s="2">
+      <c r="I124" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B125" s="1" t="s">
         <v>290</v>
@@ -5016,16 +4902,13 @@
       <c r="H125" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I125" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J125" s="2">
+      <c r="I125" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>290</v>
@@ -5042,16 +4925,13 @@
       <c r="H126" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I126" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J126" s="2">
+      <c r="I126" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>290</v>
@@ -5068,16 +4948,13 @@
       <c r="H127" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I127" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J127" s="2">
+      <c r="I127" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>290</v>
@@ -5094,16 +4971,13 @@
       <c r="H128" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I128" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J128" s="2">
+      <c r="I128" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>290</v>
@@ -5120,16 +4994,13 @@
       <c r="H129" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I129" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J129" s="2">
+      <c r="I129" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B130" s="1" t="s">
         <v>290</v>
@@ -5146,16 +5017,13 @@
       <c r="H130" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I130" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J130" s="2">
+      <c r="I130" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>290</v>
@@ -5172,16 +5040,13 @@
       <c r="H131" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I131" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J131" s="2">
+      <c r="I131" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>290</v>
@@ -5198,16 +5063,13 @@
       <c r="H132" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I132" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J132" s="2">
+      <c r="I132" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>290</v>
@@ -5224,16 +5086,13 @@
       <c r="H133" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I133" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J133" s="2">
+      <c r="I133" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>290</v>
@@ -5250,16 +5109,13 @@
       <c r="H134" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I134" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J134" s="2">
+      <c r="I134" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>290</v>
@@ -5276,16 +5132,13 @@
       <c r="H135" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I135" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J135" s="2">
+      <c r="I135" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>290</v>
@@ -5302,16 +5155,13 @@
       <c r="H136" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I136" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J136" s="2">
+      <c r="I136" s="2">
         <v>45109</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>290</v>
@@ -5328,16 +5178,13 @@
       <c r="H137" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I137" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J137" s="2">
+      <c r="I137" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>290</v>
@@ -5354,16 +5201,13 @@
       <c r="H138" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I138" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J138" s="2">
+      <c r="I138" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>290</v>
@@ -5380,16 +5224,13 @@
       <c r="H139" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I139" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J139" s="2">
+      <c r="I139" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>290</v>
@@ -5406,16 +5247,13 @@
       <c r="H140" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I140" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J140" s="2">
+      <c r="I140" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>290</v>
@@ -5432,16 +5270,13 @@
       <c r="H141" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I141" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J141" s="2">
+      <c r="I141" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>290</v>
@@ -5458,16 +5293,13 @@
       <c r="H142" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I142" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J142" s="2">
+      <c r="I142" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>290</v>
@@ -5484,16 +5316,13 @@
       <c r="H143" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I143" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J143" s="2">
+      <c r="I143" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>290</v>
@@ -5510,16 +5339,13 @@
       <c r="H144" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I144" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J144" s="2">
+      <c r="I144" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>290</v>
@@ -5536,16 +5362,13 @@
       <c r="H145" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I145" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J145" s="2">
+      <c r="I145" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>290</v>
@@ -5562,16 +5385,13 @@
       <c r="H146" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I146" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J146" s="2">
+      <c r="I146" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>290</v>
@@ -5588,16 +5408,13 @@
       <c r="H147" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I147" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J147" s="2">
+      <c r="I147" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>290</v>
@@ -5614,16 +5431,13 @@
       <c r="H148" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I148" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J148" s="2">
+      <c r="I148" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>290</v>
@@ -5640,16 +5454,13 @@
       <c r="H149" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I149" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J149" s="2">
+      <c r="I149" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>290</v>
@@ -5666,16 +5477,13 @@
       <c r="H150" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I150" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J150" s="2">
+      <c r="I150" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>290</v>
@@ -5692,16 +5500,13 @@
       <c r="H151" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I151" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J151" s="2">
+      <c r="I151" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>290</v>
@@ -5718,16 +5523,13 @@
       <c r="H152" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I152" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J152" s="2">
+      <c r="I152" s="2">
         <v>45110</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>290</v>
@@ -5744,16 +5546,13 @@
       <c r="H153" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I153" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J153" s="2">
+      <c r="I153" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>290</v>
@@ -5770,16 +5569,13 @@
       <c r="H154" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I154" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J154" s="2">
+      <c r="I154" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>290</v>
@@ -5796,16 +5592,13 @@
       <c r="H155" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I155" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J155" s="2">
+      <c r="I155" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>290</v>
@@ -5822,16 +5615,13 @@
       <c r="H156" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I156" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J156" s="2">
+      <c r="I156" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>290</v>
@@ -5848,16 +5638,13 @@
       <c r="H157" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I157" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J157" s="2">
+      <c r="I157" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>290</v>
@@ -5874,16 +5661,13 @@
       <c r="H158" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I158" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J158" s="2">
+      <c r="I158" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B159" s="1" t="s">
         <v>290</v>
@@ -5900,16 +5684,13 @@
       <c r="H159" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I159" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J159" s="2">
+      <c r="I159" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B160" s="1" t="s">
         <v>290</v>
@@ -5926,16 +5707,13 @@
       <c r="H160" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I160" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="J160" s="2">
+      <c r="I160" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>290</v>
@@ -5952,16 +5730,13 @@
       <c r="H161" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I161" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J161" s="2">
+      <c r="I161" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>290</v>
@@ -5978,16 +5753,13 @@
       <c r="H162" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I162" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J162" s="2">
+      <c r="I162" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B163" s="1" t="s">
         <v>290</v>
@@ -6004,16 +5776,13 @@
       <c r="H163" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I163" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J163" s="2">
+      <c r="I163" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>290</v>
@@ -6030,16 +5799,13 @@
       <c r="H164" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I164" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J164" s="2">
+      <c r="I164" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>290</v>
@@ -6056,16 +5822,13 @@
       <c r="H165" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I165" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J165" s="2">
+      <c r="I165" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="B166" s="1" t="s">
         <v>290</v>
@@ -6082,16 +5845,13 @@
       <c r="H166" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I166" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J166" s="2">
+      <c r="I166" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B167" s="1" t="s">
         <v>290</v>
@@ -6108,16 +5868,13 @@
       <c r="H167" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I167" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J167" s="2">
+      <c r="I167" s="2">
         <v>45111</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B168" s="1" t="s">
         <v>290</v>
@@ -6134,10 +5891,7 @@
       <c r="H168" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I168" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J168" s="2">
+      <c r="I168" s="2">
         <v>45111</v>
       </c>
     </row>

</xml_diff>